<commit_message>
wire more endpoints, actually
</commit_message>
<xml_diff>
--- a/docs/data/tables/company_summaries.xlsx
+++ b/docs/data/tables/company_summaries.xlsx
@@ -569,244 +569,244 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Walmart</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C2" t="n">
-        <v>5504.92</v>
+        <v>14049.66</v>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="E2" t="n">
-        <v>143.8</v>
+        <v>3249.6</v>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="G2" t="n">
-        <v>30</v>
+        <v>1691.4</v>
       </c>
       <c r="H2" t="n">
+        <v>7</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1168.8</v>
+      </c>
+      <c r="J2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K2" t="n">
+        <v>389.4</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M2" t="n">
+        <v>2190</v>
+      </c>
+      <c r="N2" t="n">
         <v>1</v>
       </c>
-      <c r="I2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K2" t="n">
-        <v>103.8</v>
-      </c>
-      <c r="L2" t="n">
-        <v>18</v>
-      </c>
-      <c r="M2" t="n">
-        <v>1843.12</v>
-      </c>
-      <c r="N2" t="n">
-        <v>5</v>
-      </c>
       <c r="O2" t="n">
-        <v>828</v>
+        <v>90</v>
       </c>
       <c r="P2" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>942.96</v>
+        <v>200</v>
       </c>
       <c r="R2" t="n">
         <v>2</v>
       </c>
       <c r="S2" t="n">
-        <v>72.16</v>
+        <v>1900</v>
       </c>
       <c r="T2" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="U2" t="n">
-        <v>3518</v>
+        <v>8610.060000000001</v>
       </c>
       <c r="V2" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="W2" t="n">
-        <v>2111.34</v>
+        <v>7810.06</v>
       </c>
       <c r="X2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="Y2" t="n">
-        <v>1086.66</v>
+        <v>340</v>
       </c>
       <c r="Z2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AA2" t="n">
-        <v>320</v>
+        <v>460</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Walmart</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="C3" t="n">
-        <v>14049.66</v>
+        <v>5504.92</v>
       </c>
       <c r="D3" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>3249.6</v>
+        <v>143.8</v>
       </c>
       <c r="F3" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G3" t="n">
-        <v>1691.4</v>
+        <v>30</v>
       </c>
       <c r="H3" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>1168.8</v>
+        <v>10</v>
       </c>
       <c r="J3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K3" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="L3" t="n">
+        <v>18</v>
+      </c>
+      <c r="M3" t="n">
+        <v>1843.12</v>
+      </c>
+      <c r="N3" t="n">
         <v>5</v>
       </c>
-      <c r="K3" t="n">
-        <v>389.4</v>
-      </c>
-      <c r="L3" t="n">
-        <v>4</v>
-      </c>
-      <c r="M3" t="n">
-        <v>2190</v>
-      </c>
-      <c r="N3" t="n">
-        <v>1</v>
-      </c>
       <c r="O3" t="n">
-        <v>90</v>
+        <v>828</v>
       </c>
       <c r="P3" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="Q3" t="n">
-        <v>200</v>
+        <v>942.96</v>
       </c>
       <c r="R3" t="n">
         <v>2</v>
       </c>
       <c r="S3" t="n">
-        <v>1900</v>
+        <v>72.16</v>
       </c>
       <c r="T3" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="U3" t="n">
-        <v>8610.060000000001</v>
+        <v>3518</v>
       </c>
       <c r="V3" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="W3" t="n">
-        <v>7810.06</v>
+        <v>2111.34</v>
       </c>
       <c r="X3" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="Y3" t="n">
-        <v>340</v>
+        <v>1086.66</v>
       </c>
       <c r="Z3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AA3" t="n">
-        <v>460</v>
+        <v>320</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Exxon Mobil</t>
+          <t>Tractor Supply</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>87</v>
+        <v>53</v>
       </c>
       <c r="C4" t="n">
-        <v>51944.2</v>
+        <v>14088</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E4" t="n">
-        <v>2872</v>
+        <v>666</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>1150</v>
+        <v>445</v>
       </c>
       <c r="H4" t="n">
         <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>1722</v>
+        <v>80</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>141</v>
       </c>
       <c r="L4" t="n">
-        <v>81</v>
+        <v>40</v>
       </c>
       <c r="M4" t="n">
-        <v>48732.2</v>
+        <v>13212</v>
       </c>
       <c r="N4" t="n">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="O4" t="n">
-        <v>38654.74000000001</v>
+        <v>10702</v>
       </c>
       <c r="P4" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="Q4" t="n">
-        <v>7670.58</v>
+        <v>1934</v>
       </c>
       <c r="R4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S4" t="n">
-        <v>2406.88</v>
+        <v>576</v>
       </c>
       <c r="T4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U4" t="n">
-        <v>340</v>
+        <v>210</v>
       </c>
       <c r="V4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W4" t="n">
-        <v>340</v>
+        <v>210</v>
       </c>
       <c r="X4" t="n">
         <v>0</v>
@@ -824,74 +824,74 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tractor Supply</t>
+          <t>Exxon Mobil</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>53</v>
+        <v>87</v>
       </c>
       <c r="C5" t="n">
-        <v>14088</v>
+        <v>51944.2</v>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>666</v>
+        <v>2872</v>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>445</v>
+        <v>1150</v>
       </c>
       <c r="H5" t="n">
         <v>2</v>
       </c>
       <c r="I5" t="n">
-        <v>80</v>
+        <v>1722</v>
       </c>
       <c r="J5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>141</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>40</v>
+        <v>81</v>
       </c>
       <c r="M5" t="n">
-        <v>13212</v>
+        <v>48732.2</v>
       </c>
       <c r="N5" t="n">
-        <v>22</v>
+        <v>62</v>
       </c>
       <c r="O5" t="n">
-        <v>10702</v>
+        <v>38654.74000000001</v>
       </c>
       <c r="P5" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="Q5" t="n">
-        <v>1934</v>
+        <v>7670.58</v>
       </c>
       <c r="R5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S5" t="n">
-        <v>576</v>
+        <v>2406.88</v>
       </c>
       <c r="T5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U5" t="n">
-        <v>210</v>
+        <v>340</v>
       </c>
       <c r="V5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W5" t="n">
-        <v>210</v>
+        <v>340</v>
       </c>
       <c r="X5" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
copy updates? extra endpoints?
</commit_message>
<xml_diff>
--- a/docs/data/tables/company_summaries.xlsx
+++ b/docs/data/tables/company_summaries.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA5"/>
+  <dimension ref="A1:AA6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,86 +569,86 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Lockheed Martin</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C2" t="n">
-        <v>14049.66</v>
+        <v>11146.24</v>
       </c>
       <c r="D2" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E2" t="n">
-        <v>3249.6</v>
+        <v>6594</v>
       </c>
       <c r="F2" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="G2" t="n">
-        <v>1691.4</v>
+        <v>5881</v>
       </c>
       <c r="H2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I2" t="n">
-        <v>1168.8</v>
+        <v>580</v>
       </c>
       <c r="J2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K2" t="n">
-        <v>389.4</v>
+        <v>133</v>
       </c>
       <c r="L2" t="n">
         <v>4</v>
       </c>
       <c r="M2" t="n">
-        <v>2190</v>
+        <v>817.5</v>
       </c>
       <c r="N2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O2" t="n">
+        <v>567.5</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>2</v>
+      </c>
+      <c r="S2" t="n">
+        <v>250</v>
+      </c>
+      <c r="T2" t="n">
+        <v>28</v>
+      </c>
+      <c r="U2" t="n">
+        <v>3734.74</v>
+      </c>
+      <c r="V2" t="n">
+        <v>25</v>
+      </c>
+      <c r="W2" t="n">
+        <v>3522.34</v>
+      </c>
+      <c r="X2" t="n">
         <v>1</v>
       </c>
-      <c r="O2" t="n">
-        <v>90</v>
-      </c>
-      <c r="P2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>200</v>
-      </c>
-      <c r="R2" t="n">
-        <v>2</v>
-      </c>
-      <c r="S2" t="n">
-        <v>1900</v>
-      </c>
-      <c r="T2" t="n">
-        <v>41</v>
-      </c>
-      <c r="U2" t="n">
-        <v>8610.060000000001</v>
-      </c>
-      <c r="V2" t="n">
-        <v>30</v>
-      </c>
-      <c r="W2" t="n">
-        <v>7810.06</v>
-      </c>
-      <c r="X2" t="n">
-        <v>6</v>
-      </c>
       <c r="Y2" t="n">
-        <v>340</v>
+        <v>70</v>
       </c>
       <c r="Z2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AA2" t="n">
-        <v>460</v>
+        <v>142.4</v>
       </c>
     </row>
     <row r="3">
@@ -661,7 +661,7 @@
         <v>62</v>
       </c>
       <c r="C3" t="n">
-        <v>5504.92</v>
+        <v>5504.919999999999</v>
       </c>
       <c r="D3" t="n">
         <v>6</v>
@@ -739,86 +739,86 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tractor Supply</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="C4" t="n">
-        <v>14088</v>
+        <v>14049.66</v>
       </c>
       <c r="D4" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="E4" t="n">
-        <v>666</v>
+        <v>3249.6</v>
       </c>
       <c r="F4" t="n">
+        <v>14</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1691.4</v>
+      </c>
+      <c r="H4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1168.8</v>
+      </c>
+      <c r="J4" t="n">
         <v>5</v>
       </c>
-      <c r="G4" t="n">
-        <v>445</v>
-      </c>
-      <c r="H4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I4" t="n">
-        <v>80</v>
-      </c>
-      <c r="J4" t="n">
-        <v>3</v>
-      </c>
       <c r="K4" t="n">
-        <v>141</v>
+        <v>389.4</v>
       </c>
       <c r="L4" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="M4" t="n">
-        <v>13212</v>
+        <v>2190</v>
       </c>
       <c r="N4" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="O4" t="n">
-        <v>10702</v>
+        <v>90</v>
       </c>
       <c r="P4" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>1934</v>
+        <v>200</v>
       </c>
       <c r="R4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="S4" t="n">
-        <v>576</v>
+        <v>1900</v>
       </c>
       <c r="T4" t="n">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="U4" t="n">
-        <v>210</v>
+        <v>8610.060000000001</v>
       </c>
       <c r="V4" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="W4" t="n">
-        <v>210</v>
+        <v>7810.06</v>
       </c>
       <c r="X4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Y4" t="n">
-        <v>0</v>
+        <v>340</v>
       </c>
       <c r="Z4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AA4" t="n">
-        <v>0</v>
+        <v>460</v>
       </c>
     </row>
     <row r="5">
@@ -867,7 +867,7 @@
         <v>62</v>
       </c>
       <c r="O5" t="n">
-        <v>38654.74000000001</v>
+        <v>38654.74</v>
       </c>
       <c r="P5" t="n">
         <v>13</v>
@@ -903,6 +903,91 @@
         <v>0</v>
       </c>
       <c r="AA5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tractor Supply</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>53</v>
+      </c>
+      <c r="C6" t="n">
+        <v>14088</v>
+      </c>
+      <c r="D6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" t="n">
+        <v>666</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>445</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>80</v>
+      </c>
+      <c r="J6" t="n">
+        <v>3</v>
+      </c>
+      <c r="K6" t="n">
+        <v>141</v>
+      </c>
+      <c r="L6" t="n">
+        <v>40</v>
+      </c>
+      <c r="M6" t="n">
+        <v>13212</v>
+      </c>
+      <c r="N6" t="n">
+        <v>22</v>
+      </c>
+      <c r="O6" t="n">
+        <v>10702</v>
+      </c>
+      <c r="P6" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1934</v>
+      </c>
+      <c r="R6" t="n">
+        <v>7</v>
+      </c>
+      <c r="S6" t="n">
+        <v>576</v>
+      </c>
+      <c r="T6" t="n">
+        <v>3</v>
+      </c>
+      <c r="U6" t="n">
+        <v>210</v>
+      </c>
+      <c r="V6" t="n">
+        <v>3</v>
+      </c>
+      <c r="W6" t="n">
+        <v>210</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -917,7 +1002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA5"/>
+  <dimension ref="A1:AA6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1060,340 +1145,425 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Walmart</t>
+          <t>Lockheed Martin</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>200</v>
       </c>
       <c r="C2" t="n">
-        <v>5504.92</v>
+        <v>11146.24</v>
       </c>
       <c r="D2" t="n">
-        <v>22</v>
+        <v>120</v>
       </c>
       <c r="E2" t="n">
-        <v>143.8</v>
+        <v>6648</v>
       </c>
       <c r="F2" t="n">
+        <v>96</v>
+      </c>
+      <c r="G2" t="n">
+        <v>5935</v>
+      </c>
+      <c r="H2" t="n">
+        <v>14</v>
+      </c>
+      <c r="I2" t="n">
+        <v>580</v>
+      </c>
+      <c r="J2" t="n">
+        <v>10</v>
+      </c>
+      <c r="K2" t="n">
+        <v>133</v>
+      </c>
+      <c r="L2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M2" t="n">
+        <v>884.16</v>
+      </c>
+      <c r="N2" t="n">
         <v>6</v>
       </c>
-      <c r="G2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J2" t="n">
-        <v>14</v>
-      </c>
-      <c r="K2" t="n">
-        <v>103.8</v>
-      </c>
-      <c r="L2" t="n">
-        <v>58</v>
-      </c>
-      <c r="M2" t="n">
-        <v>2003.1</v>
-      </c>
-      <c r="N2" t="n">
-        <v>16</v>
-      </c>
       <c r="O2" t="n">
-        <v>948</v>
+        <v>634.16</v>
       </c>
       <c r="P2" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>982.9400000000001</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S2" t="n">
-        <v>72.16</v>
+        <v>250</v>
       </c>
       <c r="T2" t="n">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="U2" t="n">
-        <v>3358.02</v>
+        <v>3614.08</v>
       </c>
       <c r="V2" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="W2" t="n">
-        <v>1991.34</v>
+        <v>3401.68</v>
       </c>
       <c r="X2" t="n">
-        <v>42</v>
+        <v>2</v>
       </c>
       <c r="Y2" t="n">
-        <v>1046.68</v>
+        <v>70</v>
       </c>
       <c r="Z2" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AA2" t="n">
-        <v>320.0000000000001</v>
+        <v>142.4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Walmart</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>200</v>
       </c>
       <c r="C3" t="n">
-        <v>14049.66</v>
+        <v>5504.92</v>
       </c>
       <c r="D3" t="n">
-        <v>98</v>
+        <v>22</v>
       </c>
       <c r="E3" t="n">
-        <v>3249.6</v>
+        <v>143.8</v>
       </c>
       <c r="F3" t="n">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="G3" t="n">
-        <v>1691.4</v>
+        <v>30</v>
       </c>
       <c r="H3" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="I3" t="n">
-        <v>1168.8</v>
+        <v>10</v>
       </c>
       <c r="J3" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="K3" t="n">
-        <v>389.4</v>
+        <v>103.8</v>
       </c>
       <c r="L3" t="n">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="M3" t="n">
-        <v>2190</v>
+        <v>2003.1</v>
       </c>
       <c r="N3" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="O3" t="n">
-        <v>90</v>
+        <v>948</v>
       </c>
       <c r="P3" t="n">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="Q3" t="n">
-        <v>200</v>
+        <v>982.9399999999999</v>
       </c>
       <c r="R3" t="n">
         <v>6</v>
       </c>
       <c r="S3" t="n">
-        <v>1900</v>
+        <v>72.16</v>
       </c>
       <c r="T3" t="n">
-        <v>92</v>
+        <v>120</v>
       </c>
       <c r="U3" t="n">
-        <v>8610.060000000001</v>
+        <v>3358.02</v>
       </c>
       <c r="V3" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="W3" t="n">
-        <v>7810.06</v>
+        <v>1991.34</v>
       </c>
       <c r="X3" t="n">
+        <v>42</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>1046.68</v>
+      </c>
+      <c r="Z3" t="n">
         <v>12</v>
       </c>
-      <c r="Y3" t="n">
-        <v>340</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>10</v>
-      </c>
       <c r="AA3" t="n">
-        <v>460</v>
+        <v>320.0000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Exxon Mobil</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>200</v>
       </c>
       <c r="C4" t="n">
-        <v>51944.2</v>
+        <v>14049.66</v>
       </c>
       <c r="D4" t="n">
-        <v>24</v>
+        <v>98</v>
       </c>
       <c r="E4" t="n">
-        <v>2402</v>
+        <v>3249.6</v>
       </c>
       <c r="F4" t="n">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="G4" t="n">
-        <v>1180</v>
+        <v>1691.4</v>
       </c>
       <c r="H4" t="n">
+        <v>28</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1168.8</v>
+      </c>
+      <c r="J4" t="n">
+        <v>22</v>
+      </c>
+      <c r="K4" t="n">
+        <v>389.4</v>
+      </c>
+      <c r="L4" t="n">
         <v>10</v>
       </c>
-      <c r="I4" t="n">
-        <v>1222</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>162</v>
-      </c>
       <c r="M4" t="n">
-        <v>48709.7</v>
+        <v>2190</v>
       </c>
       <c r="N4" t="n">
-        <v>124</v>
+        <v>2</v>
       </c>
       <c r="O4" t="n">
-        <v>38632.24000000001</v>
+        <v>90</v>
       </c>
       <c r="P4" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="Q4" t="n">
-        <v>7670.58</v>
+        <v>200</v>
       </c>
       <c r="R4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S4" t="n">
+        <v>1900</v>
+      </c>
+      <c r="T4" t="n">
+        <v>92</v>
+      </c>
+      <c r="U4" t="n">
+        <v>8610.060000000001</v>
+      </c>
+      <c r="V4" t="n">
+        <v>70</v>
+      </c>
+      <c r="W4" t="n">
+        <v>7810.059999999999</v>
+      </c>
+      <c r="X4" t="n">
         <v>12</v>
       </c>
-      <c r="S4" t="n">
-        <v>2406.88</v>
-      </c>
-      <c r="T4" t="n">
-        <v>14</v>
-      </c>
-      <c r="U4" t="n">
-        <v>832.5</v>
-      </c>
-      <c r="V4" t="n">
-        <v>12</v>
-      </c>
-      <c r="W4" t="n">
-        <v>332.5</v>
-      </c>
-      <c r="X4" t="n">
-        <v>2</v>
-      </c>
       <c r="Y4" t="n">
-        <v>500</v>
+        <v>340</v>
       </c>
       <c r="Z4" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AA4" t="n">
-        <v>0</v>
+        <v>460</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tractor Supply</t>
+          <t>Exxon Mobil</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>200</v>
       </c>
       <c r="C5" t="n">
-        <v>14088</v>
+        <v>51944.2</v>
       </c>
       <c r="D5" t="n">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="E5" t="n">
-        <v>666</v>
+        <v>2402</v>
       </c>
       <c r="F5" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="G5" t="n">
-        <v>445</v>
+        <v>1180</v>
       </c>
       <c r="H5" t="n">
         <v>10</v>
       </c>
       <c r="I5" t="n">
+        <v>1222</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>162</v>
+      </c>
+      <c r="M5" t="n">
+        <v>48709.7</v>
+      </c>
+      <c r="N5" t="n">
+        <v>124</v>
+      </c>
+      <c r="O5" t="n">
+        <v>38632.24000000001</v>
+      </c>
+      <c r="P5" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>7670.58</v>
+      </c>
+      <c r="R5" t="n">
+        <v>12</v>
+      </c>
+      <c r="S5" t="n">
+        <v>2406.88</v>
+      </c>
+      <c r="T5" t="n">
+        <v>14</v>
+      </c>
+      <c r="U5" t="n">
+        <v>832.5</v>
+      </c>
+      <c r="V5" t="n">
+        <v>12</v>
+      </c>
+      <c r="W5" t="n">
+        <v>332.5</v>
+      </c>
+      <c r="X5" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>500</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tractor Supply</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>200</v>
+      </c>
+      <c r="C6" t="n">
+        <v>14088</v>
+      </c>
+      <c r="D6" t="n">
+        <v>54</v>
+      </c>
+      <c r="E6" t="n">
+        <v>666</v>
+      </c>
+      <c r="F6" t="n">
+        <v>32</v>
+      </c>
+      <c r="G6" t="n">
+        <v>445</v>
+      </c>
+      <c r="H6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" t="n">
         <v>80</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J6" t="n">
         <v>12</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K6" t="n">
         <v>141</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L6" t="n">
         <v>136</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M6" t="n">
         <v>11182</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N6" t="n">
         <v>84</v>
       </c>
-      <c r="O5" t="n">
+      <c r="O6" t="n">
         <v>8672</v>
       </c>
-      <c r="P5" t="n">
+      <c r="P6" t="n">
         <v>30</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="Q6" t="n">
         <v>1934</v>
       </c>
-      <c r="R5" t="n">
+      <c r="R6" t="n">
         <v>22</v>
       </c>
-      <c r="S5" t="n">
+      <c r="S6" t="n">
         <v>576</v>
       </c>
-      <c r="T5" t="n">
+      <c r="T6" t="n">
         <v>10</v>
       </c>
-      <c r="U5" t="n">
+      <c r="U6" t="n">
         <v>2240</v>
       </c>
-      <c r="V5" t="n">
+      <c r="V6" t="n">
         <v>10</v>
       </c>
-      <c r="W5" t="n">
+      <c r="W6" t="n">
         <v>2240</v>
       </c>
-      <c r="X5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA5" t="n">
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
improve views and plots
</commit_message>
<xml_diff>
--- a/docs/data/tables/company_summaries.xlsx
+++ b/docs/data/tables/company_summaries.xlsx
@@ -569,171 +569,171 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lockheed Martin</t>
+          <t>Walmart</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C2" t="n">
-        <v>11146.24</v>
+        <v>5504.92</v>
       </c>
       <c r="D2" t="n">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="E2" t="n">
-        <v>6594</v>
+        <v>143.8</v>
       </c>
       <c r="F2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="L2" t="n">
+        <v>18</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1843.12</v>
+      </c>
+      <c r="N2" t="n">
+        <v>5</v>
+      </c>
+      <c r="O2" t="n">
+        <v>828</v>
+      </c>
+      <c r="P2" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>942.96</v>
+      </c>
+      <c r="R2" t="n">
+        <v>2</v>
+      </c>
+      <c r="S2" t="n">
+        <v>72.16</v>
+      </c>
+      <c r="T2" t="n">
+        <v>38</v>
+      </c>
+      <c r="U2" t="n">
+        <v>3518</v>
+      </c>
+      <c r="V2" t="n">
         <v>21</v>
       </c>
-      <c r="G2" t="n">
-        <v>5881</v>
-      </c>
-      <c r="H2" t="n">
-        <v>5</v>
-      </c>
-      <c r="I2" t="n">
-        <v>580</v>
-      </c>
-      <c r="J2" t="n">
-        <v>3</v>
-      </c>
-      <c r="K2" t="n">
-        <v>133</v>
-      </c>
-      <c r="L2" t="n">
-        <v>4</v>
-      </c>
-      <c r="M2" t="n">
-        <v>817.5</v>
-      </c>
-      <c r="N2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O2" t="n">
-        <v>567.5</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>2</v>
-      </c>
-      <c r="S2" t="n">
-        <v>250</v>
-      </c>
-      <c r="T2" t="n">
-        <v>28</v>
-      </c>
-      <c r="U2" t="n">
-        <v>3734.74</v>
-      </c>
-      <c r="V2" t="n">
-        <v>25</v>
-      </c>
       <c r="W2" t="n">
-        <v>3522.34</v>
+        <v>2111.34</v>
       </c>
       <c r="X2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="Y2" t="n">
-        <v>70</v>
+        <v>1086.66</v>
       </c>
       <c r="Z2" t="n">
         <v>2</v>
       </c>
       <c r="AA2" t="n">
-        <v>142.4</v>
+        <v>320</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Walmart</t>
+          <t>Lockheed Martin</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C3" t="n">
-        <v>5504.919999999999</v>
+        <v>11146.24</v>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="E3" t="n">
-        <v>143.8</v>
+        <v>6594</v>
       </c>
       <c r="F3" t="n">
+        <v>21</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5881</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>580</v>
+      </c>
+      <c r="J3" t="n">
         <v>3</v>
       </c>
-      <c r="G3" t="n">
-        <v>30</v>
-      </c>
-      <c r="H3" t="n">
+      <c r="K3" t="n">
+        <v>133</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4</v>
+      </c>
+      <c r="M3" t="n">
+        <v>817.5</v>
+      </c>
+      <c r="N3" t="n">
+        <v>2</v>
+      </c>
+      <c r="O3" t="n">
+        <v>567.5</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>2</v>
+      </c>
+      <c r="S3" t="n">
+        <v>250</v>
+      </c>
+      <c r="T3" t="n">
+        <v>28</v>
+      </c>
+      <c r="U3" t="n">
+        <v>3734.74</v>
+      </c>
+      <c r="V3" t="n">
+        <v>25</v>
+      </c>
+      <c r="W3" t="n">
+        <v>3522.34</v>
+      </c>
+      <c r="X3" t="n">
         <v>1</v>
       </c>
-      <c r="I3" t="n">
-        <v>10</v>
-      </c>
-      <c r="J3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K3" t="n">
-        <v>103.8</v>
-      </c>
-      <c r="L3" t="n">
-        <v>18</v>
-      </c>
-      <c r="M3" t="n">
-        <v>1843.12</v>
-      </c>
-      <c r="N3" t="n">
-        <v>5</v>
-      </c>
-      <c r="O3" t="n">
-        <v>828</v>
-      </c>
-      <c r="P3" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>942.96</v>
-      </c>
-      <c r="R3" t="n">
-        <v>2</v>
-      </c>
-      <c r="S3" t="n">
-        <v>72.16</v>
-      </c>
-      <c r="T3" t="n">
-        <v>38</v>
-      </c>
-      <c r="U3" t="n">
-        <v>3518</v>
-      </c>
-      <c r="V3" t="n">
-        <v>21</v>
-      </c>
-      <c r="W3" t="n">
-        <v>2111.34</v>
-      </c>
-      <c r="X3" t="n">
-        <v>15</v>
-      </c>
       <c r="Y3" t="n">
-        <v>1086.66</v>
+        <v>70</v>
       </c>
       <c r="Z3" t="n">
         <v>2</v>
       </c>
       <c r="AA3" t="n">
-        <v>320</v>
+        <v>142.4</v>
       </c>
     </row>
     <row r="4">
@@ -867,7 +867,7 @@
         <v>62</v>
       </c>
       <c r="O5" t="n">
-        <v>38654.74</v>
+        <v>38654.74000000001</v>
       </c>
       <c r="P5" t="n">
         <v>13</v>

</xml_diff>

<commit_message>
Move SQL tab before Source in nav
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data/tables/company_summaries.xlsx
+++ b/docs/data/tables/company_summaries.xlsx
@@ -569,256 +569,256 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Walmart</t>
+          <t>Lockheed Martin</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C2" t="n">
-        <v>5504.92</v>
+        <v>11146.24</v>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="E2" t="n">
-        <v>143.8</v>
+        <v>6594</v>
       </c>
       <c r="F2" t="n">
+        <v>21</v>
+      </c>
+      <c r="G2" t="n">
+        <v>5881</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>580</v>
+      </c>
+      <c r="J2" t="n">
         <v>3</v>
       </c>
-      <c r="G2" t="n">
-        <v>30</v>
-      </c>
-      <c r="H2" t="n">
+      <c r="K2" t="n">
+        <v>133</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M2" t="n">
+        <v>817.5</v>
+      </c>
+      <c r="N2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O2" t="n">
+        <v>567.5</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>2</v>
+      </c>
+      <c r="S2" t="n">
+        <v>250</v>
+      </c>
+      <c r="T2" t="n">
+        <v>28</v>
+      </c>
+      <c r="U2" t="n">
+        <v>3734.74</v>
+      </c>
+      <c r="V2" t="n">
+        <v>25</v>
+      </c>
+      <c r="W2" t="n">
+        <v>3522.34</v>
+      </c>
+      <c r="X2" t="n">
         <v>1</v>
       </c>
-      <c r="I2" t="n">
-        <v>10</v>
-      </c>
-      <c r="J2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K2" t="n">
-        <v>103.8</v>
-      </c>
-      <c r="L2" t="n">
-        <v>18</v>
-      </c>
-      <c r="M2" t="n">
-        <v>1843.12</v>
-      </c>
-      <c r="N2" t="n">
-        <v>5</v>
-      </c>
-      <c r="O2" t="n">
-        <v>828</v>
-      </c>
-      <c r="P2" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>942.96</v>
-      </c>
-      <c r="R2" t="n">
-        <v>2</v>
-      </c>
-      <c r="S2" t="n">
-        <v>72.16</v>
-      </c>
-      <c r="T2" t="n">
-        <v>38</v>
-      </c>
-      <c r="U2" t="n">
-        <v>3518</v>
-      </c>
-      <c r="V2" t="n">
-        <v>21</v>
-      </c>
-      <c r="W2" t="n">
-        <v>2111.34</v>
-      </c>
-      <c r="X2" t="n">
-        <v>15</v>
-      </c>
       <c r="Y2" t="n">
-        <v>1086.66</v>
+        <v>70</v>
       </c>
       <c r="Z2" t="n">
         <v>2</v>
       </c>
       <c r="AA2" t="n">
-        <v>320</v>
+        <v>142.4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Lockheed Martin</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="C3" t="n">
-        <v>11146.24</v>
+        <v>14049.66</v>
       </c>
       <c r="D3" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E3" t="n">
-        <v>6594</v>
+        <v>3249.6</v>
       </c>
       <c r="F3" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G3" t="n">
-        <v>5881</v>
+        <v>1691.4</v>
       </c>
       <c r="H3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1168.8</v>
+      </c>
+      <c r="J3" t="n">
         <v>5</v>
       </c>
-      <c r="I3" t="n">
-        <v>580</v>
-      </c>
-      <c r="J3" t="n">
-        <v>3</v>
-      </c>
       <c r="K3" t="n">
-        <v>133</v>
+        <v>389.4</v>
       </c>
       <c r="L3" t="n">
         <v>4</v>
       </c>
       <c r="M3" t="n">
-        <v>817.5</v>
+        <v>2190</v>
       </c>
       <c r="N3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O3" t="n">
-        <v>567.5</v>
+        <v>90</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="R3" t="n">
         <v>2</v>
       </c>
       <c r="S3" t="n">
-        <v>250</v>
+        <v>1900</v>
       </c>
       <c r="T3" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="U3" t="n">
-        <v>3734.74</v>
+        <v>8610.060000000001</v>
       </c>
       <c r="V3" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="W3" t="n">
-        <v>3522.34</v>
+        <v>7810.06</v>
       </c>
       <c r="X3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Y3" t="n">
-        <v>70</v>
+        <v>340</v>
       </c>
       <c r="Z3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AA3" t="n">
-        <v>142.4</v>
+        <v>460</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Walmart</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="C4" t="n">
-        <v>14049.66</v>
+        <v>5504.92</v>
       </c>
       <c r="D4" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="E4" t="n">
-        <v>3249.6</v>
+        <v>143.8</v>
       </c>
       <c r="F4" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G4" t="n">
-        <v>1691.4</v>
+        <v>30</v>
       </c>
       <c r="H4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>1168.8</v>
+        <v>10</v>
       </c>
       <c r="J4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="L4" t="n">
+        <v>18</v>
+      </c>
+      <c r="M4" t="n">
+        <v>1843.12</v>
+      </c>
+      <c r="N4" t="n">
         <v>5</v>
       </c>
-      <c r="K4" t="n">
-        <v>389.4</v>
-      </c>
-      <c r="L4" t="n">
-        <v>4</v>
-      </c>
-      <c r="M4" t="n">
-        <v>2190</v>
-      </c>
-      <c r="N4" t="n">
-        <v>1</v>
-      </c>
       <c r="O4" t="n">
-        <v>90</v>
+        <v>828</v>
       </c>
       <c r="P4" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="Q4" t="n">
-        <v>200</v>
+        <v>942.96</v>
       </c>
       <c r="R4" t="n">
         <v>2</v>
       </c>
       <c r="S4" t="n">
-        <v>1900</v>
+        <v>72.16</v>
       </c>
       <c r="T4" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="U4" t="n">
-        <v>8610.060000000001</v>
+        <v>3518</v>
       </c>
       <c r="V4" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="W4" t="n">
-        <v>7810.06</v>
+        <v>2111.34</v>
       </c>
       <c r="X4" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="Y4" t="n">
-        <v>340</v>
+        <v>1086.66</v>
       </c>
       <c r="Z4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AA4" t="n">
-        <v>460</v>
+        <v>320</v>
       </c>
     </row>
     <row r="5">
@@ -867,7 +867,7 @@
         <v>62</v>
       </c>
       <c r="O5" t="n">
-        <v>38654.74000000001</v>
+        <v>38654.74</v>
       </c>
       <c r="P5" t="n">
         <v>13</v>

</xml_diff>